<commit_message>
làm app hiệp hội và bổ sung chức năng cho CRM
</commit_message>
<xml_diff>
--- a/document/TIEN_DO_CONG_VIEC_TOAN_DIEN_VIONE_MOI.xlsx
+++ b/document/TIEN_DO_CONG_VIEC_TOAN_DIEN_VIONE_MOI.xlsx
@@ -7,13 +7,15 @@
     <sheet sheetId="1" name="Tổng Quan Dự Án" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Tiến Độ Chi Tiết Chức Năng" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Kiểm Toán API Ngoài" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Web Landing" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="App ViOne Giao Diện 2" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1310" uniqueCount="556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2106" uniqueCount="876">
   <si>
     <t>BÁO CÁO TIẾN ĐỘ THỰC HIỆN TOÀN DIỆN DỰ ÁN HỆ SINH THÁI VIONE</t>
   </si>
@@ -1681,13 +1683,973 @@
   </si>
   <si>
     <t>Đăng ký Paid Apps Agreement với Apple và Google, tạo mã sản phẩm IAP và tích hợp StoreKit.</t>
+  </si>
+  <si>
+    <t>BẢNG THEO DÕI TIẾN ĐỘ &amp; HIỆN TRẠNG CÁC TRANG WEB LANDING HỆ SINH THÁI VIONE</t>
+  </si>
+  <si>
+    <t>Giao Diện Landing</t>
+  </si>
+  <si>
+    <t>Tên Section / Khối Giao Diện</t>
+  </si>
+  <si>
+    <t>Nội Dung / Bản Demo Text &amp; UI Hiện Có</t>
+  </si>
+  <si>
+    <t>Đặc Tính Kỹ Thuật &amp; Hiệu Ứng</t>
+  </si>
+  <si>
+    <t>Tích Hợp API / Biểu Mẫu</t>
+  </si>
+  <si>
+    <t>Ngày Bắt Đầu</t>
+  </si>
+  <si>
+    <t>File Nguồn Code</t>
+  </si>
+  <si>
+    <t>WBS-LAND-001</t>
+  </si>
+  <si>
+    <t>CEO 1983 Landing (Hoàng Kim)</t>
+  </si>
+  <si>
+    <t>Hero Banner Hoàng Kim CEO 1983</t>
+  </si>
+  <si>
+    <t>Khẩu hiệu "Hội tụ Tinh hoa - Kết nối Bền vững", số lượng hội viên thời gian thực, nút Đăng ký &amp; Tải App</t>
+  </si>
+  <si>
+    <t>Golden Glow gradient, hạt ánh sáng vàng chuyển động, 3D emblem xoay nhẹ</t>
+  </si>
+  <si>
+    <t>Có (Đếm hội viên active)</t>
+  </si>
+  <si>
+    <t>Hoàn thành UI &amp; Text Demo</t>
+  </si>
+  <si>
+    <t>Ceo1983Landing.tsx</t>
+  </si>
+  <si>
+    <t>WBS-LAND-002</t>
+  </si>
+  <si>
+    <t>Tôn Chỉ &amp; Giá Trị Cốt Lõi CLB</t>
+  </si>
+  <si>
+    <t>5 giá trị cốt lõi: Đoàn kết, Tương trợ, Tiên phong, Bền vững, Nghĩa tình doanh nhân sinh năm Quý Hợi 1983</t>
+  </si>
+  <si>
+    <t>Card kính tối màu mờ viền dát vàng 24K, hover phóng to nhẹ nhàng</t>
+  </si>
+  <si>
+    <t>Không (Nội dung tĩnh)</t>
+  </si>
+  <si>
+    <t>WBS-LAND-003</t>
+  </si>
+  <si>
+    <t>Ban Chấp Hành &amp; Hội Đồng Cố Vấn</t>
+  </si>
+  <si>
+    <t>Chân dung Chủ tịch, các Phó Chủ tịch chuyên trách, Trưởng ban kèm thông tin doanh nghiệp đại diện</t>
+  </si>
+  <si>
+    <t>Avatar frame kim loại vàng óng, hiệu ứng spotlight khi di chuột</t>
+  </si>
+  <si>
+    <t>Có (Đọc danh sách BCH từ CRM)</t>
+  </si>
+  <si>
+    <t>WBS-LAND-004</t>
+  </si>
+  <si>
+    <t>8 Đặc Quyền Hội Viên Kim Cương</t>
+  </si>
+  <si>
+    <t>Giao thương B2B nội khối, cấp Thẻ số NFC độc bản, tham gia Gala thường niên, bảo hộ thương hiệu</t>
+  </si>
+  <si>
+    <t>Grid 4 cột responsive, icon mạ vàng chuyển động lấp lánh</t>
+  </si>
+  <si>
+    <t>Không (Nội dung bản sắc)</t>
+  </si>
+  <si>
+    <t>WBS-LAND-005</t>
+  </si>
+  <si>
+    <t>Hệ Sinh Thái Số &amp; Ứng Dụng Di Động</t>
+  </si>
+  <si>
+    <t>Demo mockup màn hình App Hiệp hội trên iPhone 16 Pro Max, liên kết tải trên App Store &amp; Google Play</t>
+  </si>
+  <si>
+    <t>3D phone tilt parallax, quét tia sáng quét qua màn hình app</t>
+  </si>
+  <si>
+    <t>Không (Mockup trực quan)</t>
+  </si>
+  <si>
+    <t>WBS-LAND-006</t>
+  </si>
+  <si>
+    <t>Sự Kiện Sắp Diễn Ra &amp; Gala Thường Niên</t>
+  </si>
+  <si>
+    <t>Đại Hội Doanh Nhân CEO 1983 - Kỷ Nguyên Vươn Mình, Diễn đàn Giao thương &amp; Gala Dinner</t>
+  </si>
+  <si>
+    <t>Đồng hồ đếm ngược Countdown thời gian thực, nút giữ chỗ tức thì</t>
+  </si>
+  <si>
+    <t>Có (Lấy sự kiện từ Event DB)</t>
+  </si>
+  <si>
+    <t>WBS-LAND-007</t>
+  </si>
+  <si>
+    <t>Bản Tin &amp; Báo Chí Nói Về CEO 1983</t>
+  </si>
+  <si>
+    <t>Tin tức báo Tuổi Trẻ, VnExpress, Báo Doanh Nhân đưa tin về các hoạt động thiện nguyện và xúc tiến thương mại</t>
+  </si>
+  <si>
+    <t>Carousel tin tức tự động trượt mượt mà, bộ lọc tin mới nhất</t>
+  </si>
+  <si>
+    <t>Có (Lấy bài viết từ News module)</t>
+  </si>
+  <si>
+    <t>WBS-LAND-008</t>
+  </si>
+  <si>
+    <t>Biểu Mẫu Đăng Ký Gia Nhập Online</t>
+  </si>
+  <si>
+    <t>Form tiếp nhận thông tin: Họ tên, Năm sinh 1983, Tên doanh nghiệp, MST, Số điện thoại, Email, Chức vụ</t>
+  </si>
+  <si>
+    <t>Floating labels, validate realtime từng ô, hiệu ứng submit thành công</t>
+  </si>
+  <si>
+    <t>Có (Gửi hồ sơ vào CRM chờ duyệt)</t>
+  </si>
+  <si>
+    <t>WBS-LAND-009</t>
+  </si>
+  <si>
+    <t>Chân Trang &amp; Thông Tin Thường Trực</t>
+  </si>
+  <si>
+    <t>Trụ sở Ban Thư Ký, Hotline liên hệ 24/7, Email tiếp nhận tài trợ, Bản đồ Google Maps, Bản quyền 2026</t>
+  </si>
+  <si>
+    <t>Dark luxury footer, icon mạng xã hội hover gradient vàng</t>
+  </si>
+  <si>
+    <t>Không</t>
+  </si>
+  <si>
+    <t>WBS-LAND-010</t>
+  </si>
+  <si>
+    <t>CEO 1983 Landing (Blue-White)</t>
+  </si>
+  <si>
+    <t>Giao Diện Nhận Diện Xanh Thương Hiệu</t>
+  </si>
+  <si>
+    <t>Toàn bộ nội dung CEO 1983 chuẩn hóa trên nền xanh #2E3192 và trắng trang nhã, phục vụ quảng bá đại chúng</t>
+  </si>
+  <si>
+    <t>Tối ưu độ tương phản AAA, màu xanh CEO 1983 chuẩn brandbook</t>
+  </si>
+  <si>
+    <t>Có (Chia sẻ backend với bản Hoàng Kim)</t>
+  </si>
+  <si>
+    <t>Ceo1983BlueWhiteLanding.tsx</t>
+  </si>
+  <si>
+    <t>WBS-LAND-011</t>
+  </si>
+  <si>
+    <t>Association Public Landing</t>
+  </si>
+  <si>
+    <t>Cổng Thông Tin Công Cộng Hiệp Hội</t>
+  </si>
+  <si>
+    <t>Cổng thông tin mở cho đối tác bên ngoài tra cứu danh bạ hội viên chính thức, xác thực mã thẻ hội viên</t>
+  </si>
+  <si>
+    <t>Thanh tìm kiếm nhanh, bộ lọc doanh nghiệp theo tỉnh thành</t>
+  </si>
+  <si>
+    <t>Có (Public Directory API)</t>
+  </si>
+  <si>
+    <t>AssociationLandingView.tsx</t>
+  </si>
+  <si>
+    <t>WBS-LAND-012</t>
+  </si>
+  <si>
+    <t>ViOne Business Connect V1</t>
+  </si>
+  <si>
+    <t>Landing V1 - Flagship ViOne Connect</t>
+  </si>
+  <si>
+    <t>Giới thiệu nền tảng số kết nối giao thương B2B, danh thiếp số thông minh NFC 1 chạm, quản lý khách hàng</t>
+  </si>
+  <si>
+    <t>Video mockup nền, thanh điều hướng kính mờ tự động ẩn hiện</t>
+  </si>
+  <si>
+    <t>Có (Đăng ký dùng thử)</t>
+  </si>
+  <si>
+    <t>BusinessConnectLanding.tsx</t>
+  </si>
+  <si>
+    <t>WBS-LAND-013</t>
+  </si>
+  <si>
+    <t>ViOne Business Connect V2</t>
+  </si>
+  <si>
+    <t>Landing V2 - Dynamic Matrix Hub</t>
+  </si>
+  <si>
+    <t>Ma trận đối tác động 2.5D, mô phỏng mạng lưới doanh nghiệp đa ngành kết nối trao đổi chéo dịch vụ</t>
+  </si>
+  <si>
+    <t>Canvas mạng lưới tương tác kéo thả các node đối tác</t>
+  </si>
+  <si>
+    <t>Có (Đăng ký demo)</t>
+  </si>
+  <si>
+    <t>BusinessConnectLandingV2.tsx</t>
+  </si>
+  <si>
+    <t>WBS-LAND-014</t>
+  </si>
+  <si>
+    <t>ViOne Business Connect V3</t>
+  </si>
+  <si>
+    <t>Landing V3 - Minimalist Premium</t>
+  </si>
+  <si>
+    <t>Thiết kế tối giản theo tiêu chuẩn Thụy Sĩ (Swiss Design), tập trung câu chữ sắc bén và kiểu chữ nghệ thuật</t>
+  </si>
+  <si>
+    <t>Kinetic Typography, hiệu ứng cuộn mượt mà Smooth Scroll</t>
+  </si>
+  <si>
+    <t>Có (Form liên hệ tư vấn)</t>
+  </si>
+  <si>
+    <t>BusinessConnectLandingV3.tsx</t>
+  </si>
+  <si>
+    <t>WBS-LAND-015</t>
+  </si>
+  <si>
+    <t>ViOne Business Connect V4</t>
+  </si>
+  <si>
+    <t>Landing V4 - 3D Glassmorphism</t>
+  </si>
+  <si>
+    <t>Hiệu ứng kính mờ đa tầng hiện đại, thẻ doanh nhân 3D xoay góc tương tác theo tọa độ chuột của người dùng</t>
+  </si>
+  <si>
+    <t>Backdrop-filter blur, ánh sáng phản xạ động trên bề mặt kính</t>
+  </si>
+  <si>
+    <t>BusinessConnectLandingV4.tsx</t>
+  </si>
+  <si>
+    <t>WBS-LAND-016</t>
+  </si>
+  <si>
+    <t>ViOne Business Connect V5</t>
+  </si>
+  <si>
+    <t>Landing V5 - Neo-Brutalism &amp; Playful</t>
+  </si>
+  <si>
+    <t>Phong cách Neo-Brutalism với đường viền đen đậm, màu pastel tương phản cao, badge stickers hoạt hình sinh động</t>
+  </si>
+  <si>
+    <t>Hiệu ứng bouncy chuyển động khi click nút, stickers lắc lư</t>
+  </si>
+  <si>
+    <t>Có (Đăng ký trải nghiệm)</t>
+  </si>
+  <si>
+    <t>BusinessConnectLandingV5.tsx</t>
+  </si>
+  <si>
+    <t>WBS-LAND-017</t>
+  </si>
+  <si>
+    <t>ViOne Business Connect V6</t>
+  </si>
+  <si>
+    <t>Landing V6 - Cyberpunk Futuristic</t>
+  </si>
+  <si>
+    <t>Giao diện công nghệ tương lai với trạm chỉ huy điều khiển, màn hình radar quét doanh nghiệp, dòng lệnh terminal</t>
+  </si>
+  <si>
+    <t>Neon glow viền cyan &amp; tím, hiệu ứng gõ chữ terminal tự động</t>
+  </si>
+  <si>
+    <t>Có (Đăng ký đối tác công nghệ)</t>
+  </si>
+  <si>
+    <t>BusinessConnectLandingV6.tsx</t>
+  </si>
+  <si>
+    <t>WBS-LAND-018</t>
+  </si>
+  <si>
+    <t>ViOne Business Connect V7</t>
+  </si>
+  <si>
+    <t>Landing V7 - Executive Dark Gold Luxury</t>
+  </si>
+  <si>
+    <t>Phong cách doanh nhân thượng lưu, nền đen Obsidian huyền bí, chữ dát vàng và card kim loại Titanium</t>
+  </si>
+  <si>
+    <t>Hiệu ứng quét ánh kim loại lấp lánh (Shimmer effect)</t>
+  </si>
+  <si>
+    <t>Có (Đặt lịch tư vấn gói VIP)</t>
+  </si>
+  <si>
+    <t>BusinessConnectLandingV7.tsx</t>
+  </si>
+  <si>
+    <t>WBS-LAND-019</t>
+  </si>
+  <si>
+    <t>ViOne Business Connect V8</t>
+  </si>
+  <si>
+    <t>Landing V8 - High Conversion SaaS B2B</t>
+  </si>
+  <si>
+    <t>Giao diện tối ưu phễu chuyển đổi cho khách hàng doanh nghiệp, bảng so sánh chi tiết các gói tính năng và bảng giá</t>
+  </si>
+  <si>
+    <t>Sticky CTA bar khi cuộn qua hero, bảng giá chuyển đổi tháng/năm</t>
+  </si>
+  <si>
+    <t>Có (Chọn gói &amp; thanh toán)</t>
+  </si>
+  <si>
+    <t>BusinessConnectLandingV8.tsx</t>
+  </si>
+  <si>
+    <t>WBS-LAND-020</t>
+  </si>
+  <si>
+    <t>Interactive 3D Hubs</t>
+  </si>
+  <si>
+    <t>Showcase 3D Robot, Radar &amp; Shield Hub</t>
+  </si>
+  <si>
+    <t>Bộ 5 linh kiện tương tác cao cấp: Robot Orbital Hub, Cyber Radar Command, Security Shield, Pyramid Governance, Titanium Card</t>
+  </si>
+  <si>
+    <t>Render 3D thời gian thực với tương tác chuột, con quay hồi chuyển</t>
+  </si>
+  <si>
+    <t>Không (Module đồ họa tương tác)</t>
+  </si>
+  <si>
+    <t>RobotEcosystemOrbitalHub.tsx</t>
+  </si>
+  <si>
+    <t>BẢNG THEO DÕI TIẾN ĐỘ PHÁT TRIỂN APP VIONE GIAO DIỆN 2 (BUSINESS CONNECT)</t>
+  </si>
+  <si>
+    <t>Phân Hệ Giao Diện 2</t>
+  </si>
+  <si>
+    <t>Tên Chức Năng Chi Tiết (Giao Diện 2)</t>
+  </si>
+  <si>
+    <t>Đường Dẫn Màn Hình / Route</t>
+  </si>
+  <si>
+    <t>WBS-V2-001</t>
+  </si>
+  <si>
+    <t>B2B Moments &amp; Feeds</t>
+  </si>
+  <si>
+    <t>Bảng tin khoảnh khắc giao thương B2B</t>
+  </si>
+  <si>
+    <t>Dòng thời gian hiển thị bài viết giao thương, cơ hội hợp tác, nhu cầu tìm kiếm đối tác và deal chớp nhoáng</t>
+  </si>
+  <si>
+    <t>WBS-V2-002</t>
+  </si>
+  <si>
+    <t>Đăng tải khoảnh khắc &amp; deal kinh doanh B2B</t>
+  </si>
+  <si>
+    <t>Form tạo bài viết nhanh: đính kèm nhiều ảnh, chọn phân ngành B2B, thiết lập tỷ lệ chiết khấu cho đối tác</t>
+  </si>
+  <si>
+    <t>WBS-V2-003</t>
+  </si>
+  <si>
+    <t>Dòng thời gian đối tác cá nhân (Personal Feed)</t>
+  </si>
+  <si>
+    <t>Trang cá nhân của từng đối tác hiển thị toàn bộ lịch sử khoảnh khắc, các deal đã chốt và uy tín kinh doanh</t>
+  </si>
+  <si>
+    <t>/connect-app/moment/:personId</t>
+  </si>
+  <si>
+    <t>WBS-V2-004</t>
+  </si>
+  <si>
+    <t>Bộ lọc khoảnh khắc theo ngành nghề &amp; vị trí</t>
+  </si>
+  <si>
+    <t>Lọc nhanh bài viết theo Bất động sản, Công nghệ, Sản xuất, Bán lẻ, và khoảng cách định vị GPS gần nhất</t>
+  </si>
+  <si>
+    <t>Không (GPS Geolocation API)</t>
+  </si>
+  <si>
+    <t>/connect-app (Filter bar)</t>
+  </si>
+  <si>
+    <t>WBS-V2-005</t>
+  </si>
+  <si>
+    <t>Tương tác chuyên nghiệp (Like, Comment, Share)</t>
+  </si>
+  <si>
+    <t>Thả tim doanh nhân, bình luận trao đổi nhu cầu kinh doanh, chia sẻ deal trực tiếp vào hộp thư đối tác</t>
+  </si>
+  <si>
+    <t>/connect-app (Post interactions)</t>
+  </si>
+  <si>
+    <t>WBS-V2-006</t>
+  </si>
+  <si>
+    <t>Mạng Lưới Kết Nối B2B</t>
+  </si>
+  <si>
+    <t>Khám phá mạng lưới doanh nhân (Discovery Hub)</t>
+  </si>
+  <si>
+    <t>Khám phá danh bạ doanh nhân theo ngành nghề, vị trí địa lý, quy mô vốn và nhu cầu kết nối cung - cầu</t>
+  </si>
+  <si>
+    <t>/connect-app/network</t>
+  </si>
+  <si>
+    <t>WBS-V2-007</t>
+  </si>
+  <si>
+    <t>Thuật toán gợi ý đối tác AI Smart Matching</t>
+  </si>
+  <si>
+    <t>Đối chiếu hồ sơ năng lực và nhu cầu tìm đối tác để tự động đề xuất top 10 doanh nhân phù hợp nhất</t>
+  </si>
+  <si>
+    <t>Không (Local Matching Algorithm)</t>
+  </si>
+  <si>
+    <t>Đang hoàn thiện</t>
+  </si>
+  <si>
+    <t>Passed (Demo)</t>
+  </si>
+  <si>
+    <t>/connect-app/network (AI Match)</t>
+  </si>
+  <si>
+    <t>WBS-V2-008</t>
+  </si>
+  <si>
+    <t>Quản lý lời mời kết nối (Invitations &amp; Requests)</t>
+  </si>
+  <si>
+    <t>Tiếp nhận các yêu cầu kết nối đối tác, xem lời nhắn đính kèm, thực hiện Chấp nhận / Từ chối / Bỏ qua</t>
+  </si>
+  <si>
+    <t>/connect-app/network/requests</t>
+  </si>
+  <si>
+    <t>WBS-V2-009</t>
+  </si>
+  <si>
+    <t>Trang hồ sơ đối tác &amp; Kết nối chung (Mutuals)</t>
+  </si>
+  <si>
+    <t>Xem chi tiết profile đối tác, lịch sử học vấn, chức vụ doanh nghiệp và số lượng mối quan hệ chung</t>
+  </si>
+  <si>
+    <t>/connect-app/network/:personId</t>
+  </si>
+  <si>
+    <t>WBS-V2-010</t>
+  </si>
+  <si>
+    <t>Gắn thẻ phân loại đối tác (Tagging CRM)</t>
+  </si>
+  <si>
+    <t>Phân nhóm đối tác theo mức độ quan hệ: Khách hàng tiềm năng, Nhà cung cấp chiến lược, Đối tác VIP</t>
+  </si>
+  <si>
+    <t>/connect-app/network (Tags)</t>
+  </si>
+  <si>
+    <t>WBS-V2-011</t>
+  </si>
+  <si>
+    <t>Hộp Thư Đàm Phán E2E</t>
+  </si>
+  <si>
+    <t>Danh sách cuộc hội thoại mã hóa đầu cuối</t>
+  </si>
+  <si>
+    <t>Hộp thư tin nhắn tức thời, phân loại tin nhắn Chưa đọc / Tin đối tác VIP / Kênh thông báo hệ thống</t>
+  </si>
+  <si>
+    <t>Không (WebSocket / SSE nội bộ)</t>
+  </si>
+  <si>
+    <t>/connect-app/inbox</t>
+  </si>
+  <si>
+    <t>WBS-V2-012</t>
+  </si>
+  <si>
+    <t>Cửa sổ trò chuyện thời gian thực (E2E Chat Window)</t>
+  </si>
+  <si>
+    <t>Nhắn tin văn bản tốc độ cao, hiển thị trạng thái đang nhập (typing), trạng thái đã nhận và đã đọc</t>
+  </si>
+  <si>
+    <t>Không (WebSocket nội bộ)</t>
+  </si>
+  <si>
+    <t>/connect-app/inbox/:threadId</t>
+  </si>
+  <si>
+    <t>WBS-V2-013</t>
+  </si>
+  <si>
+    <t>Gửi tệp đính kèm văn bản &amp; hợp đồng kinh doanh</t>
+  </si>
+  <si>
+    <t>Hỗ trợ đính kèm các định dạng .pdf, .docx, .xlsx, .zip, .rar với tính năng quét an toàn tệp tin</t>
+  </si>
+  <si>
+    <t>Không (Local Storage / MinIO)</t>
+  </si>
+  <si>
+    <t>WBS-V2-014</t>
+  </si>
+  <si>
+    <t>Gửi hình ảnh chất lượng cao &amp; Đính kèm danh thiếp số</t>
+  </si>
+  <si>
+    <t>Không (Local Storage)</t>
+  </si>
+  <si>
+    <t>WBS-V2-015</t>
+  </si>
+  <si>
+    <t>Ghi âm &amp; Gửi tin nhắn thoại (Voice Memo)</t>
+  </si>
+  <si>
+    <t>Thu âm trực tiếp trên ứng dụng, phát sóng âm trực quan (waveform) và gửi tin nhắn thoại tức thì</t>
+  </si>
+  <si>
+    <t>Không (MediaRecorder Web API)</t>
+  </si>
+  <si>
+    <t>WBS-V2-016</t>
+  </si>
+  <si>
+    <t>Cuộc gọi thoại (Audio Call) 1-1 qua WebRTC</t>
+  </si>
+  <si>
+    <t>Kết nối đàm thoại âm thanh chất lượng cao trực tiếp giữa 2 doanh nhân qua chuẩn WebRTC P2P</t>
+  </si>
+  <si>
+    <t>Không (WebRTC STUN/TURN nội bộ)</t>
+  </si>
+  <si>
+    <t>Đang kiểm thử UAT</t>
+  </si>
+  <si>
+    <t>Testing P2P</t>
+  </si>
+  <si>
+    <t>/connect-app/inbox (Call modal)</t>
+  </si>
+  <si>
+    <t>WBS-V2-017</t>
+  </si>
+  <si>
+    <t>Cuộc gọi video (Video Call) chất lượng cao</t>
+  </si>
+  <si>
+    <t>Đàm phán truyền hình trực tiếp 1-1 với hình ảnh HD, chuyển đổi camera trước/sau, chia sẻ màn hình</t>
+  </si>
+  <si>
+    <t>/connect-app/inbox (Video modal)</t>
+  </si>
+  <si>
+    <t>WBS-V2-018</t>
+  </si>
+  <si>
+    <t>Lịch Giao Thương &amp; Hội Họp</t>
+  </si>
+  <si>
+    <t>Đặt lịch hẹn kết nối 1-1 (Business Meeting)</t>
+  </si>
+  <si>
+    <t>Chọn khung giờ trống của đối tác, gửi lời mời họp kèm chủ đề giao thương và địa điểm gặp mặt</t>
+  </si>
+  <si>
+    <t>/connect-app/calendar</t>
+  </si>
+  <si>
+    <t>WBS-V2-019</t>
+  </si>
+  <si>
+    <t>Tự động tạo link phòng họp trực tuyến</t>
+  </si>
+  <si>
+    <t>Hệ thống tự động sinh đường dẫn phòng họp ảo mã hóa bảo mật khi 2 bên đồng ý lịch họp trực tuyến</t>
+  </si>
+  <si>
+    <t>Không (Jitsi / WebRTC tích hợp)</t>
+  </si>
+  <si>
+    <t>WBS-V2-020</t>
+  </si>
+  <si>
+    <t>Đồng bộ lịch hẹn với Google Calendar &amp; Outlook</t>
+  </si>
+  <si>
+    <t>Xuất file .ics tiêu chuẩn hoặc đồng bộ OAuth với Google Calendar để nhắc nhở trên mọi thiết bị</t>
+  </si>
+  <si>
+    <t>Google Calendar API (Chưa OAuth prod)</t>
+  </si>
+  <si>
+    <t>80%</t>
+  </si>
+  <si>
+    <t>Chưa kết nối OAuth ngoài</t>
+  </si>
+  <si>
+    <t>Testing .ics</t>
+  </si>
+  <si>
+    <t>WBS-V2-021</t>
+  </si>
+  <si>
+    <t>Cộng Đồng &amp; Phân Ban</t>
+  </si>
+  <si>
+    <t>Trung tâm khám phá cộng đồng &amp; CLB doanh nghiệp</t>
+  </si>
+  <si>
+    <t>Danh sách các CLB ngành nghề (Bất động sản, Công nghệ, Y tế, Nữ doanh nhân, Thể thao Golf...)</t>
+  </si>
+  <si>
+    <t>/connect-app/community</t>
+  </si>
+  <si>
+    <t>WBS-V2-022</t>
+  </si>
+  <si>
+    <t>Danh bạ thành viên phân ban chuyên môn</t>
+  </si>
+  <si>
+    <t>Tra cứu thông tin liên lạc, chức danh và hồ sơ năng lực của các thành viên trong cùng phân ban</t>
+  </si>
+  <si>
+    <t>/connect-app/community/:id/members</t>
+  </si>
+  <si>
+    <t>WBS-V2-023</t>
+  </si>
+  <si>
+    <t>Lịch sự kiện &amp; Hội thảo nội bộ phân ban</t>
+  </si>
+  <si>
+    <t>Xem lịch hội thảo chia sẻ kinh nghiệm, các buổi Business Matching nội bộ và đăng ký giữ chỗ</t>
+  </si>
+  <si>
+    <t>/connect-app/community/:id/events</t>
+  </si>
+  <si>
+    <t>WBS-V2-024</t>
+  </si>
+  <si>
+    <t>Sàn cơ hội kinh doanh &amp; Chào thầu nội khối</t>
+  </si>
+  <si>
+    <t>Đăng tin tìm kiếm nhà thầu phụ, cơ hội đầu tư chung, chuyển nhượng dự án độc quyền cho hội viên</t>
+  </si>
+  <si>
+    <t>/connect-app/community/:id/opportunities</t>
+  </si>
+  <si>
+    <t>WBS-V2-025</t>
+  </si>
+  <si>
+    <t>Quy trình xét duyệt gia nhập CLB / Phân ban</t>
+  </si>
+  <si>
+    <t>Nộp hồ sơ gia nhập kèm thư giới thiệu, Ban Chủ nhiệm phân ban thẩm duyệt và kích hoạt quyền</t>
+  </si>
+  <si>
+    <t>/connect-app/community/requests</t>
+  </si>
+  <si>
+    <t>WBS-V2-026</t>
+  </si>
+  <si>
+    <t>Định Danh Số &amp; Thẻ Thông Minh</t>
+  </si>
+  <si>
+    <t>Quét danh thiếp giấy bằng AI OCR</t>
+  </si>
+  <si>
+    <t>Chụp ảnh danh thiếp vật lý, thuật toán OCR nhận diện tự động Họ tên, Chức vụ, Công ty, SĐT, Email, MST</t>
+  </si>
+  <si>
+    <t>Tesseract OCR / AI Vision nội bộ</t>
+  </si>
+  <si>
+    <t>/connect-app/card-scan</t>
+  </si>
+  <si>
+    <t>WBS-V2-027</t>
+  </si>
+  <si>
+    <t>Ghi &amp; Kích hoạt danh thiếp số vào thẻ chip NFC</t>
+  </si>
+  <si>
+    <t>Liên kết đường dẫn hồ sơ định danh số vào thẻ cứng NFC chuẩn NTAG213/215/216 chạm 1 giây</t>
+  </si>
+  <si>
+    <t>Web NFC API (Android Chrome)</t>
+  </si>
+  <si>
+    <t>Passed (NFC Android)</t>
+  </si>
+  <si>
+    <t>/connect-app/nfc-tags</t>
+  </si>
+  <si>
+    <t>WBS-V2-028</t>
+  </si>
+  <si>
+    <t>Bảng điều khiển hồ sơ doanh nhân &amp; cá nhân</t>
+  </si>
+  <si>
+    <t>Quản lý toàn bộ thông tin cá nhân, pháp nhân công ty, huy hiệu uy tín, thống kê lượt chạm thẻ NFC</t>
+  </si>
+  <si>
+    <t>/connect-app/me</t>
+  </si>
+  <si>
+    <t>WBS-V2-029</t>
+  </si>
+  <si>
+    <t>Xem &amp; Chia sẻ danh thiếp số thông minh (Smart Card)</t>
+  </si>
+  <si>
+    <t>Danh thiếp số tương tác: mã QR động, nút "Lưu danh bạ vào điện thoại" tải file .vcf tự động</t>
+  </si>
+  <si>
+    <t>Không (VCF generator nội bộ)</t>
+  </si>
+  <si>
+    <t>/connect-app/me/card</t>
+  </si>
+  <si>
+    <t>WBS-V2-030</t>
+  </si>
+  <si>
+    <t>Quản lý đa danh thiếp Multi-Cards</t>
+  </si>
+  <si>
+    <t>Tạo nhiều danh thiếp riêng biệt cho từng vai trò kinh doanh (CEO công ty A, Cố vấn quỹ B, Chủ nhiệm CLB C)</t>
+  </si>
+  <si>
+    <t>/connect-app/me/cards</t>
+  </si>
+  <si>
+    <t>WBS-V2-031</t>
+  </si>
+  <si>
+    <t>Chỉnh sửa hồ sơ cá nhân &amp; Doanh nghiệp</t>
+  </si>
+  <si>
+    <t>Cập nhật logo doanh nghiệp, thư viện ảnh sản phẩm, liên kết Zalo, Facebook, LinkedIn, TikTok</t>
+  </si>
+  <si>
+    <t>/connect-app/me/edit</t>
+  </si>
+  <si>
+    <t>WBS-V2-032</t>
+  </si>
+  <si>
+    <t>Bảo Mật &amp; Cài Đặt Tài Khoản</t>
+  </si>
+  <si>
+    <t>Cài đặt bảo mật 2 lớp 2FA (Authenticator TOTP)</t>
+  </si>
+  <si>
+    <t>Kích hoạt mã xác thực 6 số qua Google Authenticator hoặc Microsoft Authenticator bảo vệ tài khoản</t>
+  </si>
+  <si>
+    <t>Không (Chuẩn TOTP RFC 6238)</t>
+  </si>
+  <si>
+    <t>/connect-app/me/security</t>
+  </si>
+  <si>
+    <t>WBS-V2-033</t>
+  </si>
+  <si>
+    <t>Quản lý phiên đăng nhập thiết bị &amp; Thu hồi từ xa</t>
+  </si>
+  <si>
+    <t>Hiển thị danh sách thiết bị đang đăng nhập, địa chỉ IP, vị trí địa lý, nút "Đăng xuất khỏi thiết bị này"</t>
+  </si>
+  <si>
+    <t>Không (Session DB)</t>
+  </si>
+  <si>
+    <t>/connect-app/me/sessions</t>
+  </si>
+  <si>
+    <t>WBS-V2-034</t>
+  </si>
+  <si>
+    <t>Cài đặt cá nhân hóa thông minh Intel Personalization</t>
+  </si>
+  <si>
+    <t>Tùy biến thuật toán đề xuất, quyền riêng tư số điện thoại, chế độ ẩn danh khi lướt danh bạ đối tác</t>
+  </si>
+  <si>
+    <t>/connect-app/me/intel-settings</t>
+  </si>
+  <si>
+    <t>WBS-V2-035</t>
+  </si>
+  <si>
+    <t>Trung tâm thông báo đẩy &amp; Lịch hẹn (Notifications)</t>
+  </si>
+  <si>
+    <t>Tổng hợp thông báo kết nối, tin nhắn mới, lịch hẹn giao thương, phân loại thông báo theo mức độ khẩn</t>
+  </si>
+  <si>
+    <t>FCM (Bản thử nghiệm)</t>
+  </si>
+  <si>
+    <t>Passed (In-app)</t>
+  </si>
+  <si>
+    <t>/connect-app/notifications</t>
+  </si>
+  <si>
+    <t>WBS-V2-036</t>
+  </si>
+  <si>
+    <t>Trải Nghiệm Mobile Toàn Diện</t>
+  </si>
+  <si>
+    <t>Tối ưu vùng thao tác 1 tay (One-handed Thumb Zone)</t>
+  </si>
+  <si>
+    <t>Bố trí toàn bộ các nút thao tác chính, thanh điều hướng, action buttons ở nửa dưới màn hình để dễ với tới</t>
+  </si>
+  <si>
+    <t>Không (Quy chuẩn UI Mobile)</t>
+  </si>
+  <si>
+    <t>Hoàn thành UI Rule</t>
+  </si>
+  <si>
+    <t>Passed (Mobile)</t>
+  </si>
+  <si>
+    <t>Toàn bộ app giao diện 2</t>
+  </si>
+  <si>
+    <t>WBS-V2-037</t>
+  </si>
+  <si>
+    <t>Tự động tương thích Safe Area &amp; 3 phím điều hướng Android</t>
+  </si>
+  <si>
+    <t>Đẩy header lùi xuống dưới status bar và đẩy footer/khung chat lên trên 3 nút cảm ứng Android không bị che khuất</t>
+  </si>
+  <si>
+    <t>Không (CSS env safe-area insets)</t>
+  </si>
+  <si>
+    <t>WBS-V2-038</t>
+  </si>
+  <si>
+    <t>Tự động ẩn Footer / Tab bar khi bàn phím ảo hiển thị</t>
+  </si>
+  <si>
+    <t>Khi người dùng focus vào bất kỳ ô input / textarea nào, footer tự động ẩn ngay lập tức, không che bàn phím</t>
+  </si>
+  <si>
+    <t>Không (Focus event + CSS :has)</t>
+  </si>
+  <si>
+    <t>WBS-V2-039</t>
+  </si>
+  <si>
+    <t>Input tìm kiếm không có viền hover (Borderless Search)</t>
+  </si>
+  <si>
+    <t>Loại bỏ hoàn toàn viền đổi màu khi hover vào ô tìm kiếm, đảm bảo giao diện di động mượt mà không chớp viền</t>
+  </si>
+  <si>
+    <t>Không (CSS Borderless Rule)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1779,6 +2741,18 @@
       <sz val="9.5"/>
       <name val="Times New Roman"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="047857"/>
+      <sz val="9.5"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="0369A1"/>
+      <sz val="9.5"/>
+      <name val="Times New Roman"/>
+    </font>
   </fonts>
   <fills count="12">
     <fill>
@@ -1865,7 +2839,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1958,6 +2932,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -6907,4 +7893,2780 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:N22"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="34" customWidth="1"/>
+    <col min="5" max="5" width="50" customWidth="1"/>
+    <col min="6" max="6" width="32" customWidth="1"/>
+    <col min="7" max="7" width="26" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="13" customWidth="1"/>
+    <col min="13" max="13" width="22" customWidth="1"/>
+    <col min="14" max="14" width="36" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="22" t="s">
+        <v>556</v>
+      </c>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>557</v>
+      </c>
+      <c r="D2" s="23" t="s">
+        <v>558</v>
+      </c>
+      <c r="E2" s="23" t="s">
+        <v>559</v>
+      </c>
+      <c r="F2" s="23" t="s">
+        <v>560</v>
+      </c>
+      <c r="G2" s="23" t="s">
+        <v>561</v>
+      </c>
+      <c r="H2" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="I2" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="J2" s="23" t="s">
+        <v>562</v>
+      </c>
+      <c r="K2" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="L2" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="M2" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="N2" s="23" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="24">
+        <v>1</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>564</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>565</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>566</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>567</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>568</v>
+      </c>
+      <c r="G3" s="25" t="s">
+        <v>569</v>
+      </c>
+      <c r="H3" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="I3" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="J3" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="K3" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="L3" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="M3" s="35" t="s">
+        <v>570</v>
+      </c>
+      <c r="N3" s="25" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="28">
+        <v>2</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>572</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>565</v>
+      </c>
+      <c r="D4" s="29" t="s">
+        <v>573</v>
+      </c>
+      <c r="E4" s="29" t="s">
+        <v>574</v>
+      </c>
+      <c r="F4" s="29" t="s">
+        <v>575</v>
+      </c>
+      <c r="G4" s="29" t="s">
+        <v>576</v>
+      </c>
+      <c r="H4" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="I4" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="J4" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="L4" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="M4" s="37" t="s">
+        <v>570</v>
+      </c>
+      <c r="N4" s="29" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="24">
+        <v>3</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>577</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>565</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>578</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>579</v>
+      </c>
+      <c r="F5" s="25" t="s">
+        <v>580</v>
+      </c>
+      <c r="G5" s="25" t="s">
+        <v>581</v>
+      </c>
+      <c r="H5" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="I5" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="J5" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="K5" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="L5" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="M5" s="35" t="s">
+        <v>570</v>
+      </c>
+      <c r="N5" s="25" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="28">
+        <v>4</v>
+      </c>
+      <c r="B6" s="28" t="s">
+        <v>582</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>565</v>
+      </c>
+      <c r="D6" s="29" t="s">
+        <v>583</v>
+      </c>
+      <c r="E6" s="29" t="s">
+        <v>584</v>
+      </c>
+      <c r="F6" s="29" t="s">
+        <v>585</v>
+      </c>
+      <c r="G6" s="29" t="s">
+        <v>586</v>
+      </c>
+      <c r="H6" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="I6" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="J6" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="K6" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="L6" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="M6" s="37" t="s">
+        <v>570</v>
+      </c>
+      <c r="N6" s="29" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="24">
+        <v>5</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>587</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>565</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>588</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>589</v>
+      </c>
+      <c r="F7" s="25" t="s">
+        <v>590</v>
+      </c>
+      <c r="G7" s="25" t="s">
+        <v>591</v>
+      </c>
+      <c r="H7" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="I7" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="J7" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="K7" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="L7" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="M7" s="35" t="s">
+        <v>570</v>
+      </c>
+      <c r="N7" s="25" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="28">
+        <v>6</v>
+      </c>
+      <c r="B8" s="28" t="s">
+        <v>592</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>565</v>
+      </c>
+      <c r="D8" s="29" t="s">
+        <v>593</v>
+      </c>
+      <c r="E8" s="29" t="s">
+        <v>594</v>
+      </c>
+      <c r="F8" s="29" t="s">
+        <v>595</v>
+      </c>
+      <c r="G8" s="29" t="s">
+        <v>596</v>
+      </c>
+      <c r="H8" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="I8" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="J8" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="K8" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="L8" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="M8" s="37" t="s">
+        <v>570</v>
+      </c>
+      <c r="N8" s="29" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="24">
+        <v>7</v>
+      </c>
+      <c r="B9" s="24" t="s">
+        <v>597</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>565</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>598</v>
+      </c>
+      <c r="E9" s="25" t="s">
+        <v>599</v>
+      </c>
+      <c r="F9" s="25" t="s">
+        <v>600</v>
+      </c>
+      <c r="G9" s="25" t="s">
+        <v>601</v>
+      </c>
+      <c r="H9" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="I9" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="J9" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="K9" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="L9" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="M9" s="35" t="s">
+        <v>570</v>
+      </c>
+      <c r="N9" s="25" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="28">
+        <v>8</v>
+      </c>
+      <c r="B10" s="28" t="s">
+        <v>602</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>565</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>603</v>
+      </c>
+      <c r="E10" s="29" t="s">
+        <v>604</v>
+      </c>
+      <c r="F10" s="29" t="s">
+        <v>605</v>
+      </c>
+      <c r="G10" s="29" t="s">
+        <v>606</v>
+      </c>
+      <c r="H10" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="I10" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="J10" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="K10" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="L10" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="M10" s="37" t="s">
+        <v>570</v>
+      </c>
+      <c r="N10" s="29" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="24">
+        <v>9</v>
+      </c>
+      <c r="B11" s="24" t="s">
+        <v>607</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>565</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>608</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>609</v>
+      </c>
+      <c r="F11" s="25" t="s">
+        <v>610</v>
+      </c>
+      <c r="G11" s="25" t="s">
+        <v>611</v>
+      </c>
+      <c r="H11" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="I11" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="J11" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="K11" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="L11" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="M11" s="35" t="s">
+        <v>570</v>
+      </c>
+      <c r="N11" s="25" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="28">
+        <v>10</v>
+      </c>
+      <c r="B12" s="28" t="s">
+        <v>612</v>
+      </c>
+      <c r="C12" s="29" t="s">
+        <v>613</v>
+      </c>
+      <c r="D12" s="29" t="s">
+        <v>614</v>
+      </c>
+      <c r="E12" s="29" t="s">
+        <v>615</v>
+      </c>
+      <c r="F12" s="29" t="s">
+        <v>616</v>
+      </c>
+      <c r="G12" s="29" t="s">
+        <v>617</v>
+      </c>
+      <c r="H12" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="I12" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="J12" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="K12" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="L12" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="M12" s="37" t="s">
+        <v>570</v>
+      </c>
+      <c r="N12" s="29" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="24">
+        <v>11</v>
+      </c>
+      <c r="B13" s="24" t="s">
+        <v>619</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>620</v>
+      </c>
+      <c r="D13" s="25" t="s">
+        <v>621</v>
+      </c>
+      <c r="E13" s="25" t="s">
+        <v>622</v>
+      </c>
+      <c r="F13" s="25" t="s">
+        <v>623</v>
+      </c>
+      <c r="G13" s="25" t="s">
+        <v>624</v>
+      </c>
+      <c r="H13" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="I13" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="J13" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="K13" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="L13" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="M13" s="35" t="s">
+        <v>570</v>
+      </c>
+      <c r="N13" s="25" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="28">
+        <v>12</v>
+      </c>
+      <c r="B14" s="28" t="s">
+        <v>626</v>
+      </c>
+      <c r="C14" s="29" t="s">
+        <v>627</v>
+      </c>
+      <c r="D14" s="29" t="s">
+        <v>628</v>
+      </c>
+      <c r="E14" s="29" t="s">
+        <v>629</v>
+      </c>
+      <c r="F14" s="29" t="s">
+        <v>630</v>
+      </c>
+      <c r="G14" s="29" t="s">
+        <v>631</v>
+      </c>
+      <c r="H14" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="I14" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="J14" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="K14" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="L14" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="M14" s="37" t="s">
+        <v>570</v>
+      </c>
+      <c r="N14" s="29" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" s="24">
+        <v>13</v>
+      </c>
+      <c r="B15" s="24" t="s">
+        <v>633</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>634</v>
+      </c>
+      <c r="D15" s="25" t="s">
+        <v>635</v>
+      </c>
+      <c r="E15" s="25" t="s">
+        <v>636</v>
+      </c>
+      <c r="F15" s="25" t="s">
+        <v>637</v>
+      </c>
+      <c r="G15" s="25" t="s">
+        <v>638</v>
+      </c>
+      <c r="H15" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="I15" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="J15" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="K15" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="L15" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="M15" s="35" t="s">
+        <v>570</v>
+      </c>
+      <c r="N15" s="25" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="28">
+        <v>14</v>
+      </c>
+      <c r="B16" s="28" t="s">
+        <v>640</v>
+      </c>
+      <c r="C16" s="29" t="s">
+        <v>641</v>
+      </c>
+      <c r="D16" s="29" t="s">
+        <v>642</v>
+      </c>
+      <c r="E16" s="29" t="s">
+        <v>643</v>
+      </c>
+      <c r="F16" s="29" t="s">
+        <v>644</v>
+      </c>
+      <c r="G16" s="29" t="s">
+        <v>645</v>
+      </c>
+      <c r="H16" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="I16" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="J16" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="K16" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="L16" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="M16" s="37" t="s">
+        <v>570</v>
+      </c>
+      <c r="N16" s="29" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="24">
+        <v>15</v>
+      </c>
+      <c r="B17" s="24" t="s">
+        <v>647</v>
+      </c>
+      <c r="C17" s="25" t="s">
+        <v>648</v>
+      </c>
+      <c r="D17" s="25" t="s">
+        <v>649</v>
+      </c>
+      <c r="E17" s="25" t="s">
+        <v>650</v>
+      </c>
+      <c r="F17" s="25" t="s">
+        <v>651</v>
+      </c>
+      <c r="G17" s="25" t="s">
+        <v>631</v>
+      </c>
+      <c r="H17" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="I17" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="J17" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="K17" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="L17" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="M17" s="35" t="s">
+        <v>570</v>
+      </c>
+      <c r="N17" s="25" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" s="28">
+        <v>16</v>
+      </c>
+      <c r="B18" s="28" t="s">
+        <v>653</v>
+      </c>
+      <c r="C18" s="29" t="s">
+        <v>654</v>
+      </c>
+      <c r="D18" s="29" t="s">
+        <v>655</v>
+      </c>
+      <c r="E18" s="29" t="s">
+        <v>656</v>
+      </c>
+      <c r="F18" s="29" t="s">
+        <v>657</v>
+      </c>
+      <c r="G18" s="29" t="s">
+        <v>658</v>
+      </c>
+      <c r="H18" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="I18" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="J18" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="K18" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="L18" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="M18" s="37" t="s">
+        <v>570</v>
+      </c>
+      <c r="N18" s="29" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" s="24">
+        <v>17</v>
+      </c>
+      <c r="B19" s="24" t="s">
+        <v>660</v>
+      </c>
+      <c r="C19" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="D19" s="25" t="s">
+        <v>662</v>
+      </c>
+      <c r="E19" s="25" t="s">
+        <v>663</v>
+      </c>
+      <c r="F19" s="25" t="s">
+        <v>664</v>
+      </c>
+      <c r="G19" s="25" t="s">
+        <v>665</v>
+      </c>
+      <c r="H19" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="I19" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="J19" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="K19" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="L19" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="M19" s="35" t="s">
+        <v>570</v>
+      </c>
+      <c r="N19" s="25" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" s="28">
+        <v>18</v>
+      </c>
+      <c r="B20" s="28" t="s">
+        <v>667</v>
+      </c>
+      <c r="C20" s="29" t="s">
+        <v>668</v>
+      </c>
+      <c r="D20" s="29" t="s">
+        <v>669</v>
+      </c>
+      <c r="E20" s="29" t="s">
+        <v>670</v>
+      </c>
+      <c r="F20" s="29" t="s">
+        <v>671</v>
+      </c>
+      <c r="G20" s="29" t="s">
+        <v>672</v>
+      </c>
+      <c r="H20" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="I20" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="J20" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="K20" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="L20" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="M20" s="37" t="s">
+        <v>570</v>
+      </c>
+      <c r="N20" s="29" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" s="24">
+        <v>19</v>
+      </c>
+      <c r="B21" s="24" t="s">
+        <v>674</v>
+      </c>
+      <c r="C21" s="25" t="s">
+        <v>675</v>
+      </c>
+      <c r="D21" s="25" t="s">
+        <v>676</v>
+      </c>
+      <c r="E21" s="25" t="s">
+        <v>677</v>
+      </c>
+      <c r="F21" s="25" t="s">
+        <v>678</v>
+      </c>
+      <c r="G21" s="25" t="s">
+        <v>679</v>
+      </c>
+      <c r="H21" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="I21" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="J21" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="K21" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="L21" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="M21" s="35" t="s">
+        <v>570</v>
+      </c>
+      <c r="N21" s="25" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" s="28">
+        <v>20</v>
+      </c>
+      <c r="B22" s="28" t="s">
+        <v>681</v>
+      </c>
+      <c r="C22" s="29" t="s">
+        <v>682</v>
+      </c>
+      <c r="D22" s="29" t="s">
+        <v>683</v>
+      </c>
+      <c r="E22" s="29" t="s">
+        <v>684</v>
+      </c>
+      <c r="F22" s="29" t="s">
+        <v>685</v>
+      </c>
+      <c r="G22" s="29" t="s">
+        <v>686</v>
+      </c>
+      <c r="H22" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="I22" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="J22" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="K22" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="L22" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="M22" s="37" t="s">
+        <v>570</v>
+      </c>
+      <c r="N22" s="29" t="s">
+        <v>687</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:N41"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="36" customWidth="1"/>
+    <col min="5" max="5" width="50" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="13" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="14" max="14" width="36" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="22" t="s">
+        <v>688</v>
+      </c>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>689</v>
+      </c>
+      <c r="D2" s="23" t="s">
+        <v>690</v>
+      </c>
+      <c r="E2" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="G2" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="H2" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="I2" s="23" t="s">
+        <v>562</v>
+      </c>
+      <c r="J2" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="K2" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="L2" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="M2" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="N2" s="23" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="24">
+        <v>1</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>692</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>693</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>694</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>695</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="G3" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H3" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="I3" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J3" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K3" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L3" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="M3" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="N3" s="25" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="28">
+        <v>2</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>696</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>693</v>
+      </c>
+      <c r="D4" s="29" t="s">
+        <v>697</v>
+      </c>
+      <c r="E4" s="29" t="s">
+        <v>698</v>
+      </c>
+      <c r="F4" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="G4" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H4" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="I4" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K4" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="L4" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="M4" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="N4" s="29" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="24">
+        <v>3</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>699</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>693</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>700</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>701</v>
+      </c>
+      <c r="F5" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="G5" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H5" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="I5" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J5" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K5" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L5" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="M5" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="N5" s="25" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="28">
+        <v>4</v>
+      </c>
+      <c r="B6" s="28" t="s">
+        <v>703</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>693</v>
+      </c>
+      <c r="D6" s="29" t="s">
+        <v>704</v>
+      </c>
+      <c r="E6" s="29" t="s">
+        <v>705</v>
+      </c>
+      <c r="F6" s="29" t="s">
+        <v>706</v>
+      </c>
+      <c r="G6" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H6" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="I6" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J6" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K6" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="L6" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="M6" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="N6" s="29" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="24">
+        <v>5</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>708</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>693</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>709</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>710</v>
+      </c>
+      <c r="F7" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="G7" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H7" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="I7" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J7" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K7" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L7" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="M7" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="N7" s="25" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="28">
+        <v>6</v>
+      </c>
+      <c r="B8" s="28" t="s">
+        <v>712</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>713</v>
+      </c>
+      <c r="D8" s="29" t="s">
+        <v>714</v>
+      </c>
+      <c r="E8" s="29" t="s">
+        <v>715</v>
+      </c>
+      <c r="F8" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="G8" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H8" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="I8" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J8" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K8" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="L8" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="M8" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="N8" s="29" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="24">
+        <v>7</v>
+      </c>
+      <c r="B9" s="24" t="s">
+        <v>717</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>713</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>718</v>
+      </c>
+      <c r="E9" s="25" t="s">
+        <v>719</v>
+      </c>
+      <c r="F9" s="25" t="s">
+        <v>720</v>
+      </c>
+      <c r="G9" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H9" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="I9" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J9" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K9" s="34" t="s">
+        <v>412</v>
+      </c>
+      <c r="L9" s="35" t="s">
+        <v>721</v>
+      </c>
+      <c r="M9" s="24" t="s">
+        <v>722</v>
+      </c>
+      <c r="N9" s="25" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="28">
+        <v>8</v>
+      </c>
+      <c r="B10" s="28" t="s">
+        <v>724</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>713</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>725</v>
+      </c>
+      <c r="E10" s="29" t="s">
+        <v>726</v>
+      </c>
+      <c r="F10" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="G10" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H10" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="I10" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J10" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K10" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="L10" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="M10" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="N10" s="29" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="24">
+        <v>9</v>
+      </c>
+      <c r="B11" s="24" t="s">
+        <v>728</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>713</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>729</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>730</v>
+      </c>
+      <c r="F11" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H11" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="I11" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J11" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K11" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L11" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="M11" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="N11" s="25" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="28">
+        <v>10</v>
+      </c>
+      <c r="B12" s="28" t="s">
+        <v>732</v>
+      </c>
+      <c r="C12" s="29" t="s">
+        <v>713</v>
+      </c>
+      <c r="D12" s="29" t="s">
+        <v>733</v>
+      </c>
+      <c r="E12" s="29" t="s">
+        <v>734</v>
+      </c>
+      <c r="F12" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="G12" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H12" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="I12" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J12" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K12" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="L12" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="M12" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="N12" s="29" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="24">
+        <v>11</v>
+      </c>
+      <c r="B13" s="24" t="s">
+        <v>736</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>737</v>
+      </c>
+      <c r="D13" s="25" t="s">
+        <v>738</v>
+      </c>
+      <c r="E13" s="25" t="s">
+        <v>739</v>
+      </c>
+      <c r="F13" s="25" t="s">
+        <v>740</v>
+      </c>
+      <c r="G13" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H13" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="I13" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J13" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K13" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L13" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="M13" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="N13" s="25" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="28">
+        <v>12</v>
+      </c>
+      <c r="B14" s="28" t="s">
+        <v>742</v>
+      </c>
+      <c r="C14" s="29" t="s">
+        <v>737</v>
+      </c>
+      <c r="D14" s="29" t="s">
+        <v>743</v>
+      </c>
+      <c r="E14" s="29" t="s">
+        <v>744</v>
+      </c>
+      <c r="F14" s="29" t="s">
+        <v>745</v>
+      </c>
+      <c r="G14" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H14" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="I14" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J14" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K14" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="L14" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="M14" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="N14" s="29" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" s="24">
+        <v>13</v>
+      </c>
+      <c r="B15" s="24" t="s">
+        <v>747</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>737</v>
+      </c>
+      <c r="D15" s="25" t="s">
+        <v>748</v>
+      </c>
+      <c r="E15" s="25" t="s">
+        <v>749</v>
+      </c>
+      <c r="F15" s="25" t="s">
+        <v>750</v>
+      </c>
+      <c r="G15" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H15" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="I15" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J15" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K15" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L15" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="M15" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="N15" s="25" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="28">
+        <v>14</v>
+      </c>
+      <c r="B16" s="28" t="s">
+        <v>751</v>
+      </c>
+      <c r="C16" s="29" t="s">
+        <v>737</v>
+      </c>
+      <c r="D16" s="29" t="s">
+        <v>752</v>
+      </c>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29" t="s">
+        <v>753</v>
+      </c>
+      <c r="G16" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H16" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="I16" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J16" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K16" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="L16" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="M16" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="N16" s="29" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="24">
+        <v>15</v>
+      </c>
+      <c r="B17" s="24" t="s">
+        <v>754</v>
+      </c>
+      <c r="C17" s="25" t="s">
+        <v>737</v>
+      </c>
+      <c r="D17" s="25" t="s">
+        <v>755</v>
+      </c>
+      <c r="E17" s="25" t="s">
+        <v>756</v>
+      </c>
+      <c r="F17" s="25" t="s">
+        <v>757</v>
+      </c>
+      <c r="G17" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H17" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="I17" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J17" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K17" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L17" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="M17" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="N17" s="25" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" s="28">
+        <v>16</v>
+      </c>
+      <c r="B18" s="28" t="s">
+        <v>758</v>
+      </c>
+      <c r="C18" s="29" t="s">
+        <v>737</v>
+      </c>
+      <c r="D18" s="29" t="s">
+        <v>759</v>
+      </c>
+      <c r="E18" s="29" t="s">
+        <v>760</v>
+      </c>
+      <c r="F18" s="29" t="s">
+        <v>761</v>
+      </c>
+      <c r="G18" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H18" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="I18" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J18" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K18" s="36" t="s">
+        <v>239</v>
+      </c>
+      <c r="L18" s="37" t="s">
+        <v>762</v>
+      </c>
+      <c r="M18" s="28" t="s">
+        <v>763</v>
+      </c>
+      <c r="N18" s="29" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" s="24">
+        <v>17</v>
+      </c>
+      <c r="B19" s="24" t="s">
+        <v>765</v>
+      </c>
+      <c r="C19" s="25" t="s">
+        <v>737</v>
+      </c>
+      <c r="D19" s="25" t="s">
+        <v>766</v>
+      </c>
+      <c r="E19" s="25" t="s">
+        <v>767</v>
+      </c>
+      <c r="F19" s="25" t="s">
+        <v>761</v>
+      </c>
+      <c r="G19" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H19" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="I19" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J19" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K19" s="34" t="s">
+        <v>239</v>
+      </c>
+      <c r="L19" s="35" t="s">
+        <v>762</v>
+      </c>
+      <c r="M19" s="24" t="s">
+        <v>763</v>
+      </c>
+      <c r="N19" s="25" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" s="28">
+        <v>18</v>
+      </c>
+      <c r="B20" s="28" t="s">
+        <v>769</v>
+      </c>
+      <c r="C20" s="29" t="s">
+        <v>770</v>
+      </c>
+      <c r="D20" s="29" t="s">
+        <v>771</v>
+      </c>
+      <c r="E20" s="29" t="s">
+        <v>772</v>
+      </c>
+      <c r="F20" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="G20" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H20" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="I20" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J20" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K20" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="L20" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="M20" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="N20" s="29" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" s="24">
+        <v>19</v>
+      </c>
+      <c r="B21" s="24" t="s">
+        <v>774</v>
+      </c>
+      <c r="C21" s="25" t="s">
+        <v>770</v>
+      </c>
+      <c r="D21" s="25" t="s">
+        <v>775</v>
+      </c>
+      <c r="E21" s="25" t="s">
+        <v>776</v>
+      </c>
+      <c r="F21" s="25" t="s">
+        <v>777</v>
+      </c>
+      <c r="G21" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H21" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="I21" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J21" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K21" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L21" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="M21" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="N21" s="25" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" s="28">
+        <v>20</v>
+      </c>
+      <c r="B22" s="28" t="s">
+        <v>778</v>
+      </c>
+      <c r="C22" s="29" t="s">
+        <v>770</v>
+      </c>
+      <c r="D22" s="29" t="s">
+        <v>779</v>
+      </c>
+      <c r="E22" s="29" t="s">
+        <v>780</v>
+      </c>
+      <c r="F22" s="29" t="s">
+        <v>781</v>
+      </c>
+      <c r="G22" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H22" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="I22" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J22" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K22" s="36" t="s">
+        <v>782</v>
+      </c>
+      <c r="L22" s="37" t="s">
+        <v>783</v>
+      </c>
+      <c r="M22" s="28" t="s">
+        <v>784</v>
+      </c>
+      <c r="N22" s="29" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" s="24">
+        <v>21</v>
+      </c>
+      <c r="B23" s="24" t="s">
+        <v>785</v>
+      </c>
+      <c r="C23" s="25" t="s">
+        <v>786</v>
+      </c>
+      <c r="D23" s="25" t="s">
+        <v>787</v>
+      </c>
+      <c r="E23" s="25" t="s">
+        <v>788</v>
+      </c>
+      <c r="F23" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="G23" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H23" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="I23" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J23" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K23" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L23" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="M23" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="N23" s="25" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" s="28">
+        <v>22</v>
+      </c>
+      <c r="B24" s="28" t="s">
+        <v>790</v>
+      </c>
+      <c r="C24" s="29" t="s">
+        <v>786</v>
+      </c>
+      <c r="D24" s="29" t="s">
+        <v>791</v>
+      </c>
+      <c r="E24" s="29" t="s">
+        <v>792</v>
+      </c>
+      <c r="F24" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="G24" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H24" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="I24" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J24" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K24" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="L24" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="M24" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="N24" s="29" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" s="24">
+        <v>23</v>
+      </c>
+      <c r="B25" s="24" t="s">
+        <v>794</v>
+      </c>
+      <c r="C25" s="25" t="s">
+        <v>786</v>
+      </c>
+      <c r="D25" s="25" t="s">
+        <v>795</v>
+      </c>
+      <c r="E25" s="25" t="s">
+        <v>796</v>
+      </c>
+      <c r="F25" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="G25" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H25" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="I25" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J25" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K25" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L25" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="M25" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="N25" s="25" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="28">
+        <v>24</v>
+      </c>
+      <c r="B26" s="28" t="s">
+        <v>798</v>
+      </c>
+      <c r="C26" s="29" t="s">
+        <v>786</v>
+      </c>
+      <c r="D26" s="29" t="s">
+        <v>799</v>
+      </c>
+      <c r="E26" s="29" t="s">
+        <v>800</v>
+      </c>
+      <c r="F26" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="G26" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H26" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="I26" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J26" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K26" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="L26" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="M26" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="N26" s="29" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="24">
+        <v>25</v>
+      </c>
+      <c r="B27" s="24" t="s">
+        <v>802</v>
+      </c>
+      <c r="C27" s="25" t="s">
+        <v>786</v>
+      </c>
+      <c r="D27" s="25" t="s">
+        <v>803</v>
+      </c>
+      <c r="E27" s="25" t="s">
+        <v>804</v>
+      </c>
+      <c r="F27" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="G27" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H27" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="I27" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J27" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K27" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L27" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="M27" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="N27" s="25" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="28">
+        <v>26</v>
+      </c>
+      <c r="B28" s="28" t="s">
+        <v>806</v>
+      </c>
+      <c r="C28" s="29" t="s">
+        <v>807</v>
+      </c>
+      <c r="D28" s="29" t="s">
+        <v>808</v>
+      </c>
+      <c r="E28" s="29" t="s">
+        <v>809</v>
+      </c>
+      <c r="F28" s="29" t="s">
+        <v>810</v>
+      </c>
+      <c r="G28" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H28" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="I28" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J28" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K28" s="36" t="s">
+        <v>239</v>
+      </c>
+      <c r="L28" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="M28" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="N28" s="29" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="24">
+        <v>27</v>
+      </c>
+      <c r="B29" s="24" t="s">
+        <v>812</v>
+      </c>
+      <c r="C29" s="25" t="s">
+        <v>807</v>
+      </c>
+      <c r="D29" s="25" t="s">
+        <v>813</v>
+      </c>
+      <c r="E29" s="25" t="s">
+        <v>814</v>
+      </c>
+      <c r="F29" s="25" t="s">
+        <v>815</v>
+      </c>
+      <c r="G29" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H29" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="I29" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J29" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K29" s="34" t="s">
+        <v>412</v>
+      </c>
+      <c r="L29" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="M29" s="24" t="s">
+        <v>816</v>
+      </c>
+      <c r="N29" s="25" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="30" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="28">
+        <v>28</v>
+      </c>
+      <c r="B30" s="28" t="s">
+        <v>818</v>
+      </c>
+      <c r="C30" s="29" t="s">
+        <v>807</v>
+      </c>
+      <c r="D30" s="29" t="s">
+        <v>819</v>
+      </c>
+      <c r="E30" s="29" t="s">
+        <v>820</v>
+      </c>
+      <c r="F30" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="G30" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H30" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="I30" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J30" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K30" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="L30" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="M30" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="N30" s="29" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="31" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="24">
+        <v>29</v>
+      </c>
+      <c r="B31" s="24" t="s">
+        <v>822</v>
+      </c>
+      <c r="C31" s="25" t="s">
+        <v>807</v>
+      </c>
+      <c r="D31" s="25" t="s">
+        <v>823</v>
+      </c>
+      <c r="E31" s="25" t="s">
+        <v>824</v>
+      </c>
+      <c r="F31" s="25" t="s">
+        <v>825</v>
+      </c>
+      <c r="G31" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H31" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="I31" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J31" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K31" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L31" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="M31" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="N31" s="25" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="32" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" s="28">
+        <v>30</v>
+      </c>
+      <c r="B32" s="28" t="s">
+        <v>827</v>
+      </c>
+      <c r="C32" s="29" t="s">
+        <v>807</v>
+      </c>
+      <c r="D32" s="29" t="s">
+        <v>828</v>
+      </c>
+      <c r="E32" s="29" t="s">
+        <v>829</v>
+      </c>
+      <c r="F32" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="G32" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H32" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="I32" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J32" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K32" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="L32" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="M32" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="N32" s="29" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="24">
+        <v>31</v>
+      </c>
+      <c r="B33" s="24" t="s">
+        <v>831</v>
+      </c>
+      <c r="C33" s="25" t="s">
+        <v>807</v>
+      </c>
+      <c r="D33" s="25" t="s">
+        <v>832</v>
+      </c>
+      <c r="E33" s="25" t="s">
+        <v>833</v>
+      </c>
+      <c r="F33" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="G33" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H33" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="I33" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J33" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K33" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L33" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="M33" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="N33" s="25" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="34" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" s="28">
+        <v>32</v>
+      </c>
+      <c r="B34" s="28" t="s">
+        <v>835</v>
+      </c>
+      <c r="C34" s="29" t="s">
+        <v>836</v>
+      </c>
+      <c r="D34" s="29" t="s">
+        <v>837</v>
+      </c>
+      <c r="E34" s="29" t="s">
+        <v>838</v>
+      </c>
+      <c r="F34" s="29" t="s">
+        <v>839</v>
+      </c>
+      <c r="G34" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H34" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="I34" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J34" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K34" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="L34" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="M34" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="N34" s="29" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="35" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" s="24">
+        <v>33</v>
+      </c>
+      <c r="B35" s="24" t="s">
+        <v>841</v>
+      </c>
+      <c r="C35" s="25" t="s">
+        <v>836</v>
+      </c>
+      <c r="D35" s="25" t="s">
+        <v>842</v>
+      </c>
+      <c r="E35" s="25" t="s">
+        <v>843</v>
+      </c>
+      <c r="F35" s="25" t="s">
+        <v>844</v>
+      </c>
+      <c r="G35" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H35" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="I35" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J35" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K35" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L35" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="M35" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="N35" s="25" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="28">
+        <v>34</v>
+      </c>
+      <c r="B36" s="28" t="s">
+        <v>846</v>
+      </c>
+      <c r="C36" s="29" t="s">
+        <v>836</v>
+      </c>
+      <c r="D36" s="29" t="s">
+        <v>847</v>
+      </c>
+      <c r="E36" s="29" t="s">
+        <v>848</v>
+      </c>
+      <c r="F36" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="G36" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H36" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="I36" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J36" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K36" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="L36" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="M36" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="N36" s="29" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="37" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="24">
+        <v>35</v>
+      </c>
+      <c r="B37" s="24" t="s">
+        <v>850</v>
+      </c>
+      <c r="C37" s="25" t="s">
+        <v>836</v>
+      </c>
+      <c r="D37" s="25" t="s">
+        <v>851</v>
+      </c>
+      <c r="E37" s="25" t="s">
+        <v>852</v>
+      </c>
+      <c r="F37" s="25" t="s">
+        <v>853</v>
+      </c>
+      <c r="G37" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H37" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="I37" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J37" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K37" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L37" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="M37" s="24" t="s">
+        <v>854</v>
+      </c>
+      <c r="N37" s="25" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="38" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" s="28">
+        <v>36</v>
+      </c>
+      <c r="B38" s="28" t="s">
+        <v>856</v>
+      </c>
+      <c r="C38" s="29" t="s">
+        <v>857</v>
+      </c>
+      <c r="D38" s="29" t="s">
+        <v>858</v>
+      </c>
+      <c r="E38" s="29" t="s">
+        <v>859</v>
+      </c>
+      <c r="F38" s="29" t="s">
+        <v>860</v>
+      </c>
+      <c r="G38" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H38" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="I38" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J38" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K38" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="L38" s="37" t="s">
+        <v>861</v>
+      </c>
+      <c r="M38" s="28" t="s">
+        <v>862</v>
+      </c>
+      <c r="N38" s="29" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="39" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A39" s="24">
+        <v>37</v>
+      </c>
+      <c r="B39" s="24" t="s">
+        <v>864</v>
+      </c>
+      <c r="C39" s="25" t="s">
+        <v>857</v>
+      </c>
+      <c r="D39" s="25" t="s">
+        <v>865</v>
+      </c>
+      <c r="E39" s="25" t="s">
+        <v>866</v>
+      </c>
+      <c r="F39" s="25" t="s">
+        <v>867</v>
+      </c>
+      <c r="G39" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H39" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="I39" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J39" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K39" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L39" s="35" t="s">
+        <v>861</v>
+      </c>
+      <c r="M39" s="24" t="s">
+        <v>862</v>
+      </c>
+      <c r="N39" s="25" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="40" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A40" s="28">
+        <v>38</v>
+      </c>
+      <c r="B40" s="28" t="s">
+        <v>868</v>
+      </c>
+      <c r="C40" s="29" t="s">
+        <v>857</v>
+      </c>
+      <c r="D40" s="29" t="s">
+        <v>869</v>
+      </c>
+      <c r="E40" s="29" t="s">
+        <v>870</v>
+      </c>
+      <c r="F40" s="29" t="s">
+        <v>871</v>
+      </c>
+      <c r="G40" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="H40" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="I40" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J40" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K40" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="L40" s="37" t="s">
+        <v>861</v>
+      </c>
+      <c r="M40" s="28" t="s">
+        <v>862</v>
+      </c>
+      <c r="N40" s="29" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="41" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A41" s="24">
+        <v>39</v>
+      </c>
+      <c r="B41" s="24" t="s">
+        <v>872</v>
+      </c>
+      <c r="C41" s="25" t="s">
+        <v>857</v>
+      </c>
+      <c r="D41" s="25" t="s">
+        <v>873</v>
+      </c>
+      <c r="E41" s="25" t="s">
+        <v>874</v>
+      </c>
+      <c r="F41" s="25" t="s">
+        <v>875</v>
+      </c>
+      <c r="G41" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="H41" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="I41" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J41" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K41" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="L41" s="35" t="s">
+        <v>861</v>
+      </c>
+      <c r="M41" s="24" t="s">
+        <v>862</v>
+      </c>
+      <c r="N41" s="25" t="s">
+        <v>863</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>